<commit_message>
automatic update 2026-10-05 13:06:06
</commit_message>
<xml_diff>
--- a/d_testing_folder/d_historical_test_results1.xlsx
+++ b/d_testing_folder/d_historical_test_results1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="330">
   <si>
     <t>Word</t>
   </si>
@@ -1015,9 +1015,6 @@
   </si>
   <si>
     <t>Because of the privilege and authority God has given me, I give each of you this warning: Don’t think you are better than you really are. Be honest in your evaluation of yourselves, measuring yourselves by the faith God has given us.</t>
-  </si>
-  <si>
-    <t>05-Oct-26</t>
   </si>
   <si>
     <t>Concepts and Definitions</t>
@@ -1037,7 +1034,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -1405,7 +1402,7 @@
         <v>46023</v>
       </c>
       <c r="F2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1425,7 +1422,7 @@
         <v>46023</v>
       </c>
       <c r="F3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1445,7 +1442,7 @@
         <v>46023</v>
       </c>
       <c r="F4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1465,7 +1462,7 @@
         <v>46023</v>
       </c>
       <c r="F5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1482,7 +1479,7 @@
         <v>46023</v>
       </c>
       <c r="F6" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1502,7 +1499,7 @@
         <v>46023</v>
       </c>
       <c r="F7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1522,7 +1519,7 @@
         <v>46023</v>
       </c>
       <c r="F8" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1539,7 +1536,7 @@
         <v>46023</v>
       </c>
       <c r="F9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1556,7 +1553,7 @@
         <v>46023</v>
       </c>
       <c r="F10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1576,7 +1573,7 @@
         <v>46023</v>
       </c>
       <c r="F11" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1596,7 +1593,7 @@
         <v>46023</v>
       </c>
       <c r="F12" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1616,7 +1613,7 @@
         <v>46023</v>
       </c>
       <c r="F13" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1636,7 +1633,7 @@
         <v>46023</v>
       </c>
       <c r="F14" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1656,7 +1653,7 @@
         <v>46023</v>
       </c>
       <c r="F15" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1676,7 +1673,7 @@
         <v>46023</v>
       </c>
       <c r="F16" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1696,7 +1693,7 @@
         <v>46023</v>
       </c>
       <c r="F17" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1713,7 +1710,7 @@
         <v>46023</v>
       </c>
       <c r="F18" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1733,7 +1730,7 @@
         <v>46023</v>
       </c>
       <c r="F19" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1750,7 +1747,7 @@
         <v>46023</v>
       </c>
       <c r="F20" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1767,7 +1764,7 @@
         <v>46023</v>
       </c>
       <c r="F21" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1787,7 +1784,7 @@
         <v>46023</v>
       </c>
       <c r="F22" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1807,7 +1804,7 @@
         <v>46023</v>
       </c>
       <c r="F23" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1827,7 +1824,7 @@
         <v>46023</v>
       </c>
       <c r="F24" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1844,7 +1841,7 @@
         <v>46023</v>
       </c>
       <c r="F25" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1861,7 +1858,7 @@
         <v>46023</v>
       </c>
       <c r="F26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1881,7 +1878,7 @@
         <v>46023</v>
       </c>
       <c r="F27" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1898,7 +1895,7 @@
         <v>46023</v>
       </c>
       <c r="F28" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1918,7 +1915,7 @@
         <v>46023</v>
       </c>
       <c r="F29" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1935,7 +1932,7 @@
         <v>46023</v>
       </c>
       <c r="F30" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1955,7 +1952,7 @@
         <v>46023</v>
       </c>
       <c r="F31" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1975,7 +1972,7 @@
         <v>46023</v>
       </c>
       <c r="F32" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1992,7 +1989,7 @@
         <v>46023</v>
       </c>
       <c r="F33" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2012,7 +2009,7 @@
         <v>46023</v>
       </c>
       <c r="F34" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2032,7 +2029,7 @@
         <v>46023</v>
       </c>
       <c r="F35" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2049,7 +2046,7 @@
         <v>46023</v>
       </c>
       <c r="F36" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2069,7 +2066,7 @@
         <v>46023</v>
       </c>
       <c r="F37" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2086,7 +2083,7 @@
         <v>46023</v>
       </c>
       <c r="F38" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2106,7 +2103,7 @@
         <v>46023</v>
       </c>
       <c r="F39" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2126,7 +2123,7 @@
         <v>46023</v>
       </c>
       <c r="F40" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2143,7 +2140,7 @@
         <v>46023</v>
       </c>
       <c r="F41" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2163,7 +2160,7 @@
         <v>46296</v>
       </c>
       <c r="F42" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2183,7 +2180,7 @@
         <v>46023</v>
       </c>
       <c r="F43" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -2203,7 +2200,7 @@
         <v>46023</v>
       </c>
       <c r="F44" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -2223,7 +2220,7 @@
         <v>46023</v>
       </c>
       <c r="F45" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -2243,7 +2240,7 @@
         <v>46023</v>
       </c>
       <c r="F46" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2263,7 +2260,7 @@
         <v>46023</v>
       </c>
       <c r="F47" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -2283,7 +2280,7 @@
         <v>46023</v>
       </c>
       <c r="F48" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -2300,7 +2297,7 @@
         <v>46023</v>
       </c>
       <c r="F49" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2320,7 +2317,7 @@
         <v>46023</v>
       </c>
       <c r="F50" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -2340,7 +2337,7 @@
         <v>46023</v>
       </c>
       <c r="F51" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2357,7 +2354,7 @@
         <v>46023</v>
       </c>
       <c r="F52" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2374,7 +2371,7 @@
         <v>46023</v>
       </c>
       <c r="F53" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2394,7 +2391,7 @@
         <v>46023</v>
       </c>
       <c r="F54" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2414,7 +2411,7 @@
         <v>46023</v>
       </c>
       <c r="F55" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2434,7 +2431,7 @@
         <v>46023</v>
       </c>
       <c r="F56" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2451,7 +2448,7 @@
         <v>46023</v>
       </c>
       <c r="F57" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2471,7 +2468,7 @@
         <v>46023</v>
       </c>
       <c r="F58" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2491,7 +2488,7 @@
         <v>46023</v>
       </c>
       <c r="F59" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2511,7 +2508,7 @@
         <v>46023</v>
       </c>
       <c r="F60" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -2531,7 +2528,7 @@
         <v>46296</v>
       </c>
       <c r="F61" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -2551,7 +2548,7 @@
         <v>46023</v>
       </c>
       <c r="F62" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -2571,7 +2568,7 @@
         <v>46023</v>
       </c>
       <c r="F63" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -2591,7 +2588,7 @@
         <v>46023</v>
       </c>
       <c r="F64" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -2611,7 +2608,7 @@
         <v>46023</v>
       </c>
       <c r="F65" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -2631,7 +2628,7 @@
         <v>46023</v>
       </c>
       <c r="F66" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -2651,7 +2648,7 @@
         <v>46296</v>
       </c>
       <c r="F67" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -2668,7 +2665,7 @@
         <v>46023</v>
       </c>
       <c r="F68" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -2688,7 +2685,7 @@
         <v>46023</v>
       </c>
       <c r="F69" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -2708,7 +2705,7 @@
         <v>46023</v>
       </c>
       <c r="F70" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -2728,7 +2725,7 @@
         <v>46023</v>
       </c>
       <c r="F71" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -2748,7 +2745,7 @@
         <v>46023</v>
       </c>
       <c r="F72" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -2765,7 +2762,7 @@
         <v>46023</v>
       </c>
       <c r="F73" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -2785,7 +2782,7 @@
         <v>46023</v>
       </c>
       <c r="F74" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -2805,7 +2802,7 @@
         <v>46023</v>
       </c>
       <c r="F75" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -2822,7 +2819,7 @@
         <v>46023</v>
       </c>
       <c r="F76" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -2842,7 +2839,7 @@
         <v>46023</v>
       </c>
       <c r="F77" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -2862,7 +2859,7 @@
         <v>46023</v>
       </c>
       <c r="F78" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -2882,7 +2879,7 @@
         <v>46023</v>
       </c>
       <c r="F79" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -2902,7 +2899,7 @@
         <v>46023</v>
       </c>
       <c r="F80" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2922,7 +2919,7 @@
         <v>46023</v>
       </c>
       <c r="F81" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2939,7 +2936,7 @@
         <v>46023</v>
       </c>
       <c r="F82" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -2959,7 +2956,7 @@
         <v>46023</v>
       </c>
       <c r="F83" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2976,7 +2973,7 @@
         <v>46023</v>
       </c>
       <c r="F84" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -2996,7 +2993,7 @@
         <v>46023</v>
       </c>
       <c r="F85" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -3013,7 +3010,7 @@
         <v>46023</v>
       </c>
       <c r="F86" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -3030,7 +3027,7 @@
         <v>46023</v>
       </c>
       <c r="F87" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -3050,7 +3047,7 @@
         <v>46023</v>
       </c>
       <c r="F88" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -3070,7 +3067,7 @@
         <v>46023</v>
       </c>
       <c r="F89" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -3090,7 +3087,7 @@
         <v>46023</v>
       </c>
       <c r="F90" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -3110,7 +3107,7 @@
         <v>46023</v>
       </c>
       <c r="F91" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -3130,7 +3127,7 @@
         <v>46023</v>
       </c>
       <c r="F92" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -3150,7 +3147,7 @@
         <v>46023</v>
       </c>
       <c r="F93" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -3170,7 +3167,7 @@
         <v>46023</v>
       </c>
       <c r="F94" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -3190,7 +3187,7 @@
         <v>46023</v>
       </c>
       <c r="F95" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -3210,7 +3207,7 @@
         <v>46296</v>
       </c>
       <c r="F96" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -3230,7 +3227,7 @@
         <v>46023</v>
       </c>
       <c r="F97" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -3250,7 +3247,7 @@
         <v>46023</v>
       </c>
       <c r="F98" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3270,7 +3267,7 @@
         <v>46023</v>
       </c>
       <c r="F99" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3290,7 +3287,7 @@
         <v>46023</v>
       </c>
       <c r="F100" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -3310,7 +3307,7 @@
         <v>46023</v>
       </c>
       <c r="F101" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3330,7 +3327,7 @@
         <v>46023</v>
       </c>
       <c r="F102" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3350,7 +3347,7 @@
         <v>46023</v>
       </c>
       <c r="F103" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3370,7 +3367,7 @@
         <v>46296</v>
       </c>
       <c r="F104" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3390,7 +3387,7 @@
         <v>46296</v>
       </c>
       <c r="F105" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3410,7 +3407,7 @@
         <v>46023</v>
       </c>
       <c r="F106" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3430,7 +3427,7 @@
         <v>46023</v>
       </c>
       <c r="F107" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3450,7 +3447,7 @@
         <v>46023</v>
       </c>
       <c r="F108" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -3470,7 +3467,7 @@
         <v>46296</v>
       </c>
       <c r="F109" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3490,7 +3487,7 @@
         <v>46023</v>
       </c>
       <c r="F110" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -3510,7 +3507,7 @@
         <v>46023</v>
       </c>
       <c r="F111" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3530,7 +3527,7 @@
         <v>46296</v>
       </c>
       <c r="F112" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -3730,7 +3727,7 @@
         <v>46296</v>
       </c>
       <c r="F122" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -3750,7 +3747,7 @@
         <v>46296</v>
       </c>
       <c r="F123" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -3770,7 +3767,7 @@
         <v>46023</v>
       </c>
       <c r="F124" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -3790,7 +3787,7 @@
         <v>46296</v>
       </c>
       <c r="F125" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -3810,7 +3807,7 @@
         <v>46023</v>
       </c>
       <c r="F126" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -3830,7 +3827,7 @@
         <v>46023</v>
       </c>
       <c r="F127" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -3850,7 +3847,7 @@
         <v>46023</v>
       </c>
       <c r="F128" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -3870,7 +3867,7 @@
         <v>46023</v>
       </c>
       <c r="F129" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -3890,7 +3887,7 @@
         <v>46023</v>
       </c>
       <c r="F130" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -3910,7 +3907,7 @@
         <v>46023</v>
       </c>
       <c r="F131" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -3930,7 +3927,7 @@
         <v>46023</v>
       </c>
       <c r="F132" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -3950,7 +3947,7 @@
         <v>46023</v>
       </c>
       <c r="F133" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -3970,7 +3967,7 @@
         <v>46023</v>
       </c>
       <c r="F134" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -3990,7 +3987,7 @@
         <v>46023</v>
       </c>
       <c r="F135" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -4050,7 +4047,7 @@
         <v>46023</v>
       </c>
       <c r="F138" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="139" spans="1:6">
@@ -4090,7 +4087,7 @@
         <v>46295</v>
       </c>
       <c r="F140" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="141" spans="1:6">
@@ -4110,7 +4107,7 @@
         <v>46295</v>
       </c>
       <c r="F141" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -4130,7 +4127,7 @@
         <v>46295</v>
       </c>
       <c r="F142" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -4150,7 +4147,7 @@
         <v>46295</v>
       </c>
       <c r="F143" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -4170,7 +4167,7 @@
         <v>46295</v>
       </c>
       <c r="F144" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="145" spans="1:6">
@@ -4190,7 +4187,7 @@
         <v>46295</v>
       </c>
       <c r="F145" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -4210,7 +4207,7 @@
         <v>46296</v>
       </c>
       <c r="F146" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="147" spans="1:6">
@@ -4230,7 +4227,7 @@
         <v>46295</v>
       </c>
       <c r="F147" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="148" spans="1:6">
@@ -4270,7 +4267,7 @@
         <v>46296</v>
       </c>
       <c r="F149" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="150" spans="1:6">
@@ -4290,7 +4287,7 @@
         <v>46296</v>
       </c>
       <c r="F150" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="151" spans="1:6">
@@ -4310,7 +4307,7 @@
         <v>46296</v>
       </c>
       <c r="F151" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="152" spans="1:6">
@@ -4330,7 +4327,7 @@
         <v>46296</v>
       </c>
       <c r="F152" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="153" spans="1:6">
@@ -4350,7 +4347,7 @@
         <v>46296</v>
       </c>
       <c r="F153" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="154" spans="1:6">
@@ -4390,7 +4387,7 @@
         <v>46296</v>
       </c>
       <c r="F155" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -4410,7 +4407,7 @@
         <v>46296</v>
       </c>
       <c r="F156" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="157" spans="1:6">
@@ -4430,7 +4427,7 @@
         <v>46296</v>
       </c>
       <c r="F157" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="158" spans="1:6">
@@ -4450,7 +4447,7 @@
         <v>46298</v>
       </c>
       <c r="F158" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="159" spans="1:6">
@@ -4470,7 +4467,7 @@
         <v>46298</v>
       </c>
       <c r="F159" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="160" spans="1:6">
@@ -4490,7 +4487,7 @@
         <v>46298</v>
       </c>
       <c r="F160" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="161" spans="1:6">
@@ -4510,7 +4507,7 @@
         <v>46298</v>
       </c>
       <c r="F161" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="162" spans="1:6">
@@ -4530,7 +4527,7 @@
         <v>46298</v>
       </c>
       <c r="F162" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="163" spans="1:6">
@@ -4550,7 +4547,7 @@
         <v>46298</v>
       </c>
       <c r="F163" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="164" spans="1:6">
@@ -4570,7 +4567,7 @@
         <v>46298</v>
       </c>
       <c r="F164" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="165" spans="1:6">
@@ -4590,7 +4587,7 @@
         <v>46298</v>
       </c>
       <c r="F165" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="166" spans="1:6">
@@ -4623,14 +4620,14 @@
       <c r="C167">
         <v>0</v>
       </c>
-      <c r="D167" t="s">
-        <v>326</v>
-      </c>
-      <c r="E167" t="s">
-        <v>326</v>
+      <c r="D167" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E167" s="1">
+        <v>46300</v>
       </c>
       <c r="F167" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="168" spans="1:6">
@@ -4643,14 +4640,14 @@
       <c r="C168">
         <v>0</v>
       </c>
-      <c r="D168" t="s">
-        <v>326</v>
-      </c>
-      <c r="E168" t="s">
-        <v>326</v>
+      <c r="D168" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E168" s="1">
+        <v>46300</v>
       </c>
       <c r="F168" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="169" spans="1:6">
@@ -4663,14 +4660,14 @@
       <c r="C169">
         <v>0</v>
       </c>
-      <c r="D169" t="s">
-        <v>326</v>
-      </c>
-      <c r="E169" t="s">
-        <v>326</v>
+      <c r="D169" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E169" s="1">
+        <v>46300</v>
       </c>
       <c r="F169" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="170" spans="1:6">
@@ -4683,14 +4680,14 @@
       <c r="C170">
         <v>0</v>
       </c>
-      <c r="D170" t="s">
-        <v>326</v>
-      </c>
-      <c r="E170" t="s">
-        <v>326</v>
+      <c r="D170" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E170" s="1">
+        <v>46300</v>
       </c>
       <c r="F170" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="171" spans="1:6">
@@ -4703,14 +4700,14 @@
       <c r="C171">
         <v>0</v>
       </c>
-      <c r="D171" t="s">
-        <v>326</v>
-      </c>
-      <c r="E171" t="s">
-        <v>326</v>
+      <c r="D171" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E171" s="1">
+        <v>46300</v>
       </c>
       <c r="F171" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="172" spans="1:6">
@@ -4723,14 +4720,14 @@
       <c r="C172">
         <v>0</v>
       </c>
-      <c r="D172" t="s">
-        <v>326</v>
-      </c>
-      <c r="E172" t="s">
-        <v>326</v>
+      <c r="D172" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E172" s="1">
+        <v>46300</v>
       </c>
       <c r="F172" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="173" spans="1:6">
@@ -4743,11 +4740,11 @@
       <c r="C173">
         <v>0</v>
       </c>
-      <c r="D173" t="s">
-        <v>326</v>
-      </c>
-      <c r="E173" t="s">
-        <v>326</v>
+      <c r="D173" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E173" s="1">
+        <v>46300</v>
       </c>
       <c r="F173" t="s">
         <v>0</v>
@@ -4763,14 +4760,14 @@
       <c r="C174">
         <v>0</v>
       </c>
-      <c r="D174" t="s">
-        <v>326</v>
-      </c>
-      <c r="E174" t="s">
-        <v>326</v>
+      <c r="D174" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E174" s="1">
+        <v>46300</v>
       </c>
       <c r="F174" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="175" spans="1:6">
@@ -4783,14 +4780,14 @@
       <c r="C175">
         <v>0</v>
       </c>
-      <c r="D175" t="s">
-        <v>326</v>
-      </c>
-      <c r="E175" t="s">
-        <v>326</v>
+      <c r="D175" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E175" s="1">
+        <v>46300</v>
       </c>
       <c r="F175" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
automatic update 2026-10-06 15:07:13
</commit_message>
<xml_diff>
--- a/d_testing_folder/d_historical_test_results1.xlsx
+++ b/d_testing_folder/d_historical_test_results1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="338">
   <si>
     <t>Word</t>
   </si>
@@ -551,6 +551,15 @@
   </si>
   <si>
     <t>Romans 12:3</t>
+  </si>
+  <si>
+    <t>Latent</t>
+  </si>
+  <si>
+    <t>Prior</t>
+  </si>
+  <si>
+    <t>Posterior</t>
   </si>
   <si>
     <t>A mathematical function applied to a neuron’s weighted input that introduces non-linearity into a neural network. This nonlinearity enables the model to learn complex, non-linear relationships in the data. Activation functions are applied within layers during the forward pass of a neural network, transforming intermediate representations before passing them to the next layer. Activation choice affects gradient flow, training stability, and convergence speed. Poor choices can cause vanishing or exploding gradients, limiting the depth or effectiveness of the network</t>
@@ -1017,6 +1026,18 @@
     <t>Because of the privilege and authority God has given me, I give each of you this warning: Don’t think you are better than you really are. Be honest in your evaluation of yourselves, measuring yourselves by the faith God has given us.</t>
   </si>
   <si>
+    <t>Present or existing but not currently visible, active, or apparent, although capable of becoming evident or developing in the future.</t>
+  </si>
+  <si>
+    <t>A prior probability or prior distribution represents the probability assigned to an unknown parameter, hypothesis, or latent state before incorporating the current observed data or evidence. In Bayesian statistics, the prior captures existing knowledge, assumptions, or beliefs and is combined with the likelihood of the observed data to perform statistical inference. Priors may be based on historical data, domain knowledge, or deliberately weak assumptions when little previous information is available. In models such as Gaussian Mixture Models, the component mixing weights can be interpreted as prior probabilities of component membership before considering a particular observation.</t>
+  </si>
+  <si>
+    <t>A posterior probability or posterior distribution represents the probability assigned to an unknown parameter, hypothesis, or latent state after incorporating observed data or evidence. In Bayesian inference, the posterior is obtained by combining the prior distribution with the likelihood of the observed data according to Bayes' theorem and then normalizing the result. It therefore represents an updated state of knowledge given the available evidence. In a Gaussian Mixture Model, for example, the posterior component probabilities represent the estimated probabilities that a particular observation belongs to each Gaussian component after considering the observation's values.</t>
+  </si>
+  <si>
+    <t>2026-10-05</t>
+  </si>
+  <si>
     <t>Concepts and Definitions</t>
   </si>
   <si>
@@ -1027,6 +1048,9 @@
   </si>
   <si>
     <t>Quote</t>
+  </si>
+  <si>
+    <t>Concepts And Definition</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F175"/>
+  <dimension ref="A1:F178"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1390,7 +1414,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1402,7 +1426,7 @@
         <v>46023</v>
       </c>
       <c r="F2" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1410,7 +1434,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1422,7 +1446,7 @@
         <v>46023</v>
       </c>
       <c r="F3" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1430,7 +1454,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1442,7 +1466,7 @@
         <v>46023</v>
       </c>
       <c r="F4" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1450,7 +1474,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1462,7 +1486,7 @@
         <v>46023</v>
       </c>
       <c r="F5" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1479,7 +1503,7 @@
         <v>46023</v>
       </c>
       <c r="F6" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1487,7 +1511,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1499,7 +1523,7 @@
         <v>46023</v>
       </c>
       <c r="F7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1507,7 +1531,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -1519,7 +1543,7 @@
         <v>46023</v>
       </c>
       <c r="F8" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1536,7 +1560,7 @@
         <v>46023</v>
       </c>
       <c r="F9" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1553,7 +1577,7 @@
         <v>46023</v>
       </c>
       <c r="F10" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1561,7 +1585,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1573,7 +1597,7 @@
         <v>46023</v>
       </c>
       <c r="F11" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1581,7 +1605,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1593,7 +1617,7 @@
         <v>46023</v>
       </c>
       <c r="F12" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1601,7 +1625,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1613,7 +1637,7 @@
         <v>46023</v>
       </c>
       <c r="F13" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1621,7 +1645,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1633,7 +1657,7 @@
         <v>46023</v>
       </c>
       <c r="F14" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1641,7 +1665,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1653,7 +1677,7 @@
         <v>46023</v>
       </c>
       <c r="F15" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1661,7 +1685,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1673,7 +1697,7 @@
         <v>46023</v>
       </c>
       <c r="F16" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1681,7 +1705,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1693,7 +1717,7 @@
         <v>46023</v>
       </c>
       <c r="F17" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1710,7 +1734,7 @@
         <v>46023</v>
       </c>
       <c r="F18" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1718,7 +1742,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1730,7 +1754,7 @@
         <v>46023</v>
       </c>
       <c r="F19" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1747,7 +1771,7 @@
         <v>46023</v>
       </c>
       <c r="F20" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1764,7 +1788,7 @@
         <v>46023</v>
       </c>
       <c r="F21" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1772,7 +1796,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1784,7 +1808,7 @@
         <v>46023</v>
       </c>
       <c r="F22" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1792,7 +1816,7 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1804,7 +1828,7 @@
         <v>46023</v>
       </c>
       <c r="F23" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1812,7 +1836,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -1824,7 +1848,7 @@
         <v>46023</v>
       </c>
       <c r="F24" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1841,7 +1865,7 @@
         <v>46023</v>
       </c>
       <c r="F25" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1858,7 +1882,7 @@
         <v>46023</v>
       </c>
       <c r="F26" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1866,7 +1890,7 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1878,7 +1902,7 @@
         <v>46023</v>
       </c>
       <c r="F27" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1895,7 +1919,7 @@
         <v>46023</v>
       </c>
       <c r="F28" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1903,7 +1927,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -1915,7 +1939,7 @@
         <v>46023</v>
       </c>
       <c r="F29" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1932,7 +1956,7 @@
         <v>46023</v>
       </c>
       <c r="F30" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1940,7 +1964,7 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1952,7 +1976,7 @@
         <v>46023</v>
       </c>
       <c r="F31" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1960,7 +1984,7 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -1972,7 +1996,7 @@
         <v>46023</v>
       </c>
       <c r="F32" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1989,7 +2013,7 @@
         <v>46023</v>
       </c>
       <c r="F33" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1997,7 +2021,7 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -2009,7 +2033,7 @@
         <v>46023</v>
       </c>
       <c r="F34" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2017,7 +2041,7 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -2029,7 +2053,7 @@
         <v>46023</v>
       </c>
       <c r="F35" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2046,7 +2070,7 @@
         <v>46023</v>
       </c>
       <c r="F36" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2054,7 +2078,7 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -2066,7 +2090,7 @@
         <v>46023</v>
       </c>
       <c r="F37" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2083,7 +2107,7 @@
         <v>46023</v>
       </c>
       <c r="F38" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2091,7 +2115,7 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -2103,7 +2127,7 @@
         <v>46023</v>
       </c>
       <c r="F39" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2111,7 +2135,7 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -2123,7 +2147,7 @@
         <v>46023</v>
       </c>
       <c r="F40" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2140,7 +2164,7 @@
         <v>46023</v>
       </c>
       <c r="F41" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2148,7 +2172,7 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -2160,7 +2184,7 @@
         <v>46296</v>
       </c>
       <c r="F42" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2168,7 +2192,7 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -2180,7 +2204,7 @@
         <v>46023</v>
       </c>
       <c r="F43" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -2188,7 +2212,7 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -2200,7 +2224,7 @@
         <v>46023</v>
       </c>
       <c r="F44" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -2208,7 +2232,7 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C45">
         <v>0</v>
@@ -2220,7 +2244,7 @@
         <v>46023</v>
       </c>
       <c r="F45" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -2228,7 +2252,7 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -2240,7 +2264,7 @@
         <v>46023</v>
       </c>
       <c r="F46" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2248,7 +2272,7 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -2260,7 +2284,7 @@
         <v>46023</v>
       </c>
       <c r="F47" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -2268,7 +2292,7 @@
         <v>52</v>
       </c>
       <c r="B48" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -2280,7 +2304,7 @@
         <v>46023</v>
       </c>
       <c r="F48" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -2297,7 +2321,7 @@
         <v>46023</v>
       </c>
       <c r="F49" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2305,7 +2329,7 @@
         <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -2317,7 +2341,7 @@
         <v>46023</v>
       </c>
       <c r="F50" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -2325,7 +2349,7 @@
         <v>55</v>
       </c>
       <c r="B51" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -2337,7 +2361,7 @@
         <v>46023</v>
       </c>
       <c r="F51" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2354,7 +2378,7 @@
         <v>46023</v>
       </c>
       <c r="F52" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2371,7 +2395,7 @@
         <v>46023</v>
       </c>
       <c r="F53" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2379,7 +2403,7 @@
         <v>58</v>
       </c>
       <c r="B54" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C54">
         <v>0</v>
@@ -2391,7 +2415,7 @@
         <v>46023</v>
       </c>
       <c r="F54" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2399,7 +2423,7 @@
         <v>59</v>
       </c>
       <c r="B55" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C55">
         <v>0</v>
@@ -2411,7 +2435,7 @@
         <v>46023</v>
       </c>
       <c r="F55" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2419,7 +2443,7 @@
         <v>60</v>
       </c>
       <c r="B56" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C56">
         <v>0</v>
@@ -2431,7 +2455,7 @@
         <v>46023</v>
       </c>
       <c r="F56" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2448,7 +2472,7 @@
         <v>46023</v>
       </c>
       <c r="F57" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2456,7 +2480,7 @@
         <v>62</v>
       </c>
       <c r="B58" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C58">
         <v>0</v>
@@ -2468,7 +2492,7 @@
         <v>46023</v>
       </c>
       <c r="F58" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2476,7 +2500,7 @@
         <v>63</v>
       </c>
       <c r="B59" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -2488,7 +2512,7 @@
         <v>46023</v>
       </c>
       <c r="F59" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2496,7 +2520,7 @@
         <v>64</v>
       </c>
       <c r="B60" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -2508,7 +2532,7 @@
         <v>46023</v>
       </c>
       <c r="F60" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -2516,7 +2540,7 @@
         <v>65</v>
       </c>
       <c r="B61" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -2528,7 +2552,7 @@
         <v>46296</v>
       </c>
       <c r="F61" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -2536,7 +2560,7 @@
         <v>66</v>
       </c>
       <c r="B62" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -2548,7 +2572,7 @@
         <v>46023</v>
       </c>
       <c r="F62" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -2556,7 +2580,7 @@
         <v>67</v>
       </c>
       <c r="B63" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -2568,7 +2592,7 @@
         <v>46023</v>
       </c>
       <c r="F63" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -2576,7 +2600,7 @@
         <v>68</v>
       </c>
       <c r="B64" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -2588,7 +2612,7 @@
         <v>46023</v>
       </c>
       <c r="F64" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -2596,7 +2620,7 @@
         <v>69</v>
       </c>
       <c r="B65" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -2608,7 +2632,7 @@
         <v>46023</v>
       </c>
       <c r="F65" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -2616,7 +2640,7 @@
         <v>70</v>
       </c>
       <c r="B66" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -2628,7 +2652,7 @@
         <v>46023</v>
       </c>
       <c r="F66" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -2636,7 +2660,7 @@
         <v>71</v>
       </c>
       <c r="B67" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C67">
         <v>0</v>
@@ -2648,7 +2672,7 @@
         <v>46296</v>
       </c>
       <c r="F67" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -2665,7 +2689,7 @@
         <v>46023</v>
       </c>
       <c r="F68" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -2673,7 +2697,7 @@
         <v>73</v>
       </c>
       <c r="B69" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -2685,7 +2709,7 @@
         <v>46023</v>
       </c>
       <c r="F69" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -2693,7 +2717,7 @@
         <v>74</v>
       </c>
       <c r="B70" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -2705,7 +2729,7 @@
         <v>46023</v>
       </c>
       <c r="F70" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -2713,7 +2737,7 @@
         <v>75</v>
       </c>
       <c r="B71" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -2725,7 +2749,7 @@
         <v>46023</v>
       </c>
       <c r="F71" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -2733,7 +2757,7 @@
         <v>76</v>
       </c>
       <c r="B72" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C72">
         <v>0</v>
@@ -2745,7 +2769,7 @@
         <v>46023</v>
       </c>
       <c r="F72" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -2762,7 +2786,7 @@
         <v>46023</v>
       </c>
       <c r="F73" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -2770,7 +2794,7 @@
         <v>78</v>
       </c>
       <c r="B74" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C74">
         <v>0</v>
@@ -2782,7 +2806,7 @@
         <v>46023</v>
       </c>
       <c r="F74" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -2790,7 +2814,7 @@
         <v>79</v>
       </c>
       <c r="B75" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C75">
         <v>0</v>
@@ -2802,7 +2826,7 @@
         <v>46023</v>
       </c>
       <c r="F75" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -2819,7 +2843,7 @@
         <v>46023</v>
       </c>
       <c r="F76" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -2827,7 +2851,7 @@
         <v>81</v>
       </c>
       <c r="B77" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C77">
         <v>0</v>
@@ -2839,7 +2863,7 @@
         <v>46023</v>
       </c>
       <c r="F77" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -2847,7 +2871,7 @@
         <v>82</v>
       </c>
       <c r="B78" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -2859,7 +2883,7 @@
         <v>46023</v>
       </c>
       <c r="F78" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -2867,7 +2891,7 @@
         <v>83</v>
       </c>
       <c r="B79" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -2879,7 +2903,7 @@
         <v>46023</v>
       </c>
       <c r="F79" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -2887,7 +2911,7 @@
         <v>84</v>
       </c>
       <c r="B80" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C80">
         <v>0</v>
@@ -2899,7 +2923,7 @@
         <v>46023</v>
       </c>
       <c r="F80" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2907,7 +2931,7 @@
         <v>85</v>
       </c>
       <c r="B81" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C81">
         <v>0</v>
@@ -2919,7 +2943,7 @@
         <v>46023</v>
       </c>
       <c r="F81" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2936,7 +2960,7 @@
         <v>46023</v>
       </c>
       <c r="F82" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -2944,7 +2968,7 @@
         <v>87</v>
       </c>
       <c r="B83" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C83">
         <v>0</v>
@@ -2956,7 +2980,7 @@
         <v>46023</v>
       </c>
       <c r="F83" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2973,7 +2997,7 @@
         <v>46023</v>
       </c>
       <c r="F84" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -2981,7 +3005,7 @@
         <v>89</v>
       </c>
       <c r="B85" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -2993,7 +3017,7 @@
         <v>46023</v>
       </c>
       <c r="F85" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -3010,7 +3034,7 @@
         <v>46023</v>
       </c>
       <c r="F86" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -3027,7 +3051,7 @@
         <v>46023</v>
       </c>
       <c r="F87" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -3035,7 +3059,7 @@
         <v>92</v>
       </c>
       <c r="B88" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -3047,7 +3071,7 @@
         <v>46023</v>
       </c>
       <c r="F88" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -3055,7 +3079,7 @@
         <v>93</v>
       </c>
       <c r="B89" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -3067,7 +3091,7 @@
         <v>46023</v>
       </c>
       <c r="F89" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -3075,7 +3099,7 @@
         <v>94</v>
       </c>
       <c r="B90" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -3087,7 +3111,7 @@
         <v>46023</v>
       </c>
       <c r="F90" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -3095,7 +3119,7 @@
         <v>95</v>
       </c>
       <c r="B91" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -3107,7 +3131,7 @@
         <v>46023</v>
       </c>
       <c r="F91" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -3115,7 +3139,7 @@
         <v>96</v>
       </c>
       <c r="B92" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -3127,7 +3151,7 @@
         <v>46023</v>
       </c>
       <c r="F92" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -3135,7 +3159,7 @@
         <v>97</v>
       </c>
       <c r="B93" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -3147,7 +3171,7 @@
         <v>46023</v>
       </c>
       <c r="F93" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -3155,7 +3179,7 @@
         <v>98</v>
       </c>
       <c r="B94" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C94">
         <v>0</v>
@@ -3167,7 +3191,7 @@
         <v>46023</v>
       </c>
       <c r="F94" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -3175,7 +3199,7 @@
         <v>99</v>
       </c>
       <c r="B95" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C95">
         <v>0</v>
@@ -3187,7 +3211,7 @@
         <v>46023</v>
       </c>
       <c r="F95" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -3195,7 +3219,7 @@
         <v>100</v>
       </c>
       <c r="B96" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C96">
         <v>0</v>
@@ -3207,7 +3231,7 @@
         <v>46296</v>
       </c>
       <c r="F96" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -3215,7 +3239,7 @@
         <v>101</v>
       </c>
       <c r="B97" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C97">
         <v>0</v>
@@ -3227,7 +3251,7 @@
         <v>46023</v>
       </c>
       <c r="F97" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -3235,7 +3259,7 @@
         <v>102</v>
       </c>
       <c r="B98" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C98">
         <v>0</v>
@@ -3247,7 +3271,7 @@
         <v>46023</v>
       </c>
       <c r="F98" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3255,7 +3279,7 @@
         <v>103</v>
       </c>
       <c r="B99" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C99">
         <v>0</v>
@@ -3267,7 +3291,7 @@
         <v>46023</v>
       </c>
       <c r="F99" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3275,7 +3299,7 @@
         <v>104</v>
       </c>
       <c r="B100" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C100">
         <v>0</v>
@@ -3287,7 +3311,7 @@
         <v>46023</v>
       </c>
       <c r="F100" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -3295,7 +3319,7 @@
         <v>105</v>
       </c>
       <c r="B101" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C101">
         <v>0</v>
@@ -3307,7 +3331,7 @@
         <v>46023</v>
       </c>
       <c r="F101" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3315,7 +3339,7 @@
         <v>106</v>
       </c>
       <c r="B102" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C102">
         <v>0</v>
@@ -3327,7 +3351,7 @@
         <v>46023</v>
       </c>
       <c r="F102" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3335,7 +3359,7 @@
         <v>107</v>
       </c>
       <c r="B103" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C103">
         <v>0</v>
@@ -3347,7 +3371,7 @@
         <v>46023</v>
       </c>
       <c r="F103" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3355,7 +3379,7 @@
         <v>108</v>
       </c>
       <c r="B104" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C104">
         <v>0</v>
@@ -3367,7 +3391,7 @@
         <v>46296</v>
       </c>
       <c r="F104" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3375,7 +3399,7 @@
         <v>109</v>
       </c>
       <c r="B105" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C105">
         <v>0</v>
@@ -3387,7 +3411,7 @@
         <v>46296</v>
       </c>
       <c r="F105" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3395,7 +3419,7 @@
         <v>110</v>
       </c>
       <c r="B106" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C106">
         <v>0</v>
@@ -3407,7 +3431,7 @@
         <v>46023</v>
       </c>
       <c r="F106" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3415,7 +3439,7 @@
         <v>111</v>
       </c>
       <c r="B107" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C107">
         <v>0</v>
@@ -3427,7 +3451,7 @@
         <v>46023</v>
       </c>
       <c r="F107" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3435,7 +3459,7 @@
         <v>112</v>
       </c>
       <c r="B108" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -3447,7 +3471,7 @@
         <v>46023</v>
       </c>
       <c r="F108" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -3455,7 +3479,7 @@
         <v>113</v>
       </c>
       <c r="B109" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -3467,7 +3491,7 @@
         <v>46296</v>
       </c>
       <c r="F109" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3475,7 +3499,7 @@
         <v>114</v>
       </c>
       <c r="B110" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -3487,7 +3511,7 @@
         <v>46023</v>
       </c>
       <c r="F110" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -3495,7 +3519,7 @@
         <v>115</v>
       </c>
       <c r="B111" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -3507,7 +3531,7 @@
         <v>46023</v>
       </c>
       <c r="F111" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3515,7 +3539,7 @@
         <v>116</v>
       </c>
       <c r="B112" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -3527,7 +3551,7 @@
         <v>46296</v>
       </c>
       <c r="F112" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -3535,7 +3559,7 @@
         <v>117</v>
       </c>
       <c r="B113" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -3555,7 +3579,7 @@
         <v>118</v>
       </c>
       <c r="B114" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -3575,7 +3599,7 @@
         <v>119</v>
       </c>
       <c r="B115" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -3595,7 +3619,7 @@
         <v>120</v>
       </c>
       <c r="B116" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C116">
         <v>0</v>
@@ -3615,7 +3639,7 @@
         <v>121</v>
       </c>
       <c r="B117" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C117">
         <v>0</v>
@@ -3635,7 +3659,7 @@
         <v>122</v>
       </c>
       <c r="B118" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C118">
         <v>0</v>
@@ -3655,7 +3679,7 @@
         <v>123</v>
       </c>
       <c r="B119" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C119">
         <v>0</v>
@@ -3675,7 +3699,7 @@
         <v>124</v>
       </c>
       <c r="B120" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C120">
         <v>0</v>
@@ -3695,7 +3719,7 @@
         <v>125</v>
       </c>
       <c r="B121" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C121">
         <v>0</v>
@@ -3715,7 +3739,7 @@
         <v>126</v>
       </c>
       <c r="B122" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C122">
         <v>0</v>
@@ -3727,7 +3751,7 @@
         <v>46296</v>
       </c>
       <c r="F122" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -3735,7 +3759,7 @@
         <v>127</v>
       </c>
       <c r="B123" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C123">
         <v>0</v>
@@ -3747,7 +3771,7 @@
         <v>46296</v>
       </c>
       <c r="F123" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -3755,7 +3779,7 @@
         <v>128</v>
       </c>
       <c r="B124" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C124">
         <v>0</v>
@@ -3767,7 +3791,7 @@
         <v>46023</v>
       </c>
       <c r="F124" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -3775,7 +3799,7 @@
         <v>129</v>
       </c>
       <c r="B125" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C125">
         <v>0</v>
@@ -3787,7 +3811,7 @@
         <v>46296</v>
       </c>
       <c r="F125" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -3795,7 +3819,7 @@
         <v>130</v>
       </c>
       <c r="B126" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C126">
         <v>0</v>
@@ -3807,7 +3831,7 @@
         <v>46023</v>
       </c>
       <c r="F126" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -3815,7 +3839,7 @@
         <v>131</v>
       </c>
       <c r="B127" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C127">
         <v>0</v>
@@ -3827,7 +3851,7 @@
         <v>46023</v>
       </c>
       <c r="F127" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -3835,7 +3859,7 @@
         <v>132</v>
       </c>
       <c r="B128" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C128">
         <v>0</v>
@@ -3847,7 +3871,7 @@
         <v>46023</v>
       </c>
       <c r="F128" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -3855,7 +3879,7 @@
         <v>133</v>
       </c>
       <c r="B129" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C129">
         <v>0</v>
@@ -3867,7 +3891,7 @@
         <v>46023</v>
       </c>
       <c r="F129" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -3875,7 +3899,7 @@
         <v>134</v>
       </c>
       <c r="B130" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C130">
         <v>0</v>
@@ -3887,7 +3911,7 @@
         <v>46023</v>
       </c>
       <c r="F130" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -3895,7 +3919,7 @@
         <v>135</v>
       </c>
       <c r="B131" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C131">
         <v>0</v>
@@ -3907,7 +3931,7 @@
         <v>46023</v>
       </c>
       <c r="F131" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -3915,7 +3939,7 @@
         <v>136</v>
       </c>
       <c r="B132" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C132">
         <v>0</v>
@@ -3927,7 +3951,7 @@
         <v>46023</v>
       </c>
       <c r="F132" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -3935,7 +3959,7 @@
         <v>137</v>
       </c>
       <c r="B133" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C133">
         <v>0</v>
@@ -3947,7 +3971,7 @@
         <v>46023</v>
       </c>
       <c r="F133" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -3955,7 +3979,7 @@
         <v>138</v>
       </c>
       <c r="B134" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -3967,7 +3991,7 @@
         <v>46023</v>
       </c>
       <c r="F134" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -3975,7 +3999,7 @@
         <v>139</v>
       </c>
       <c r="B135" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -3987,7 +4011,7 @@
         <v>46023</v>
       </c>
       <c r="F135" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -3995,7 +4019,7 @@
         <v>140</v>
       </c>
       <c r="B136" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -4015,7 +4039,7 @@
         <v>141</v>
       </c>
       <c r="B137" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -4035,7 +4059,7 @@
         <v>142</v>
       </c>
       <c r="B138" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -4047,7 +4071,7 @@
         <v>46023</v>
       </c>
       <c r="F138" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="139" spans="1:6">
@@ -4055,7 +4079,7 @@
         <v>143</v>
       </c>
       <c r="B139" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C139">
         <v>0</v>
@@ -4075,7 +4099,7 @@
         <v>144</v>
       </c>
       <c r="B140" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -4087,7 +4111,7 @@
         <v>46295</v>
       </c>
       <c r="F140" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="141" spans="1:6">
@@ -4095,7 +4119,7 @@
         <v>145</v>
       </c>
       <c r="B141" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -4107,7 +4131,7 @@
         <v>46295</v>
       </c>
       <c r="F141" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -4115,7 +4139,7 @@
         <v>146</v>
       </c>
       <c r="B142" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -4127,7 +4151,7 @@
         <v>46295</v>
       </c>
       <c r="F142" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -4135,7 +4159,7 @@
         <v>147</v>
       </c>
       <c r="B143" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C143">
         <v>0</v>
@@ -4147,7 +4171,7 @@
         <v>46295</v>
       </c>
       <c r="F143" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -4155,7 +4179,7 @@
         <v>148</v>
       </c>
       <c r="B144" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C144">
         <v>0</v>
@@ -4167,7 +4191,7 @@
         <v>46295</v>
       </c>
       <c r="F144" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="145" spans="1:6">
@@ -4175,7 +4199,7 @@
         <v>149</v>
       </c>
       <c r="B145" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C145">
         <v>0</v>
@@ -4187,7 +4211,7 @@
         <v>46295</v>
       </c>
       <c r="F145" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -4195,7 +4219,7 @@
         <v>150</v>
       </c>
       <c r="B146" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C146">
         <v>0</v>
@@ -4207,7 +4231,7 @@
         <v>46296</v>
       </c>
       <c r="F146" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="147" spans="1:6">
@@ -4215,7 +4239,7 @@
         <v>151</v>
       </c>
       <c r="B147" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C147">
         <v>0</v>
@@ -4227,7 +4251,7 @@
         <v>46295</v>
       </c>
       <c r="F147" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="148" spans="1:6">
@@ -4235,7 +4259,7 @@
         <v>152</v>
       </c>
       <c r="B148" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C148">
         <v>0</v>
@@ -4255,7 +4279,7 @@
         <v>153</v>
       </c>
       <c r="B149" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -4267,7 +4291,7 @@
         <v>46296</v>
       </c>
       <c r="F149" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="150" spans="1:6">
@@ -4275,7 +4299,7 @@
         <v>154</v>
       </c>
       <c r="B150" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C150">
         <v>0</v>
@@ -4287,7 +4311,7 @@
         <v>46296</v>
       </c>
       <c r="F150" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="151" spans="1:6">
@@ -4295,7 +4319,7 @@
         <v>155</v>
       </c>
       <c r="B151" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C151">
         <v>0</v>
@@ -4307,7 +4331,7 @@
         <v>46296</v>
       </c>
       <c r="F151" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="152" spans="1:6">
@@ -4315,7 +4339,7 @@
         <v>156</v>
       </c>
       <c r="B152" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C152">
         <v>0</v>
@@ -4327,7 +4351,7 @@
         <v>46296</v>
       </c>
       <c r="F152" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="153" spans="1:6">
@@ -4335,7 +4359,7 @@
         <v>157</v>
       </c>
       <c r="B153" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C153">
         <v>0</v>
@@ -4347,7 +4371,7 @@
         <v>46296</v>
       </c>
       <c r="F153" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="154" spans="1:6">
@@ -4355,7 +4379,7 @@
         <v>158</v>
       </c>
       <c r="B154" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C154">
         <v>0</v>
@@ -4375,7 +4399,7 @@
         <v>159</v>
       </c>
       <c r="B155" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C155">
         <v>0</v>
@@ -4387,7 +4411,7 @@
         <v>46296</v>
       </c>
       <c r="F155" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -4395,7 +4419,7 @@
         <v>160</v>
       </c>
       <c r="B156" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -4407,7 +4431,7 @@
         <v>46296</v>
       </c>
       <c r="F156" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="157" spans="1:6">
@@ -4415,7 +4439,7 @@
         <v>161</v>
       </c>
       <c r="B157" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C157">
         <v>0</v>
@@ -4427,7 +4451,7 @@
         <v>46296</v>
       </c>
       <c r="F157" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="158" spans="1:6">
@@ -4435,7 +4459,7 @@
         <v>162</v>
       </c>
       <c r="B158" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -4447,7 +4471,7 @@
         <v>46298</v>
       </c>
       <c r="F158" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="159" spans="1:6">
@@ -4455,7 +4479,7 @@
         <v>163</v>
       </c>
       <c r="B159" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -4467,7 +4491,7 @@
         <v>46298</v>
       </c>
       <c r="F159" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="160" spans="1:6">
@@ -4475,7 +4499,7 @@
         <v>164</v>
       </c>
       <c r="B160" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C160">
         <v>0</v>
@@ -4487,7 +4511,7 @@
         <v>46298</v>
       </c>
       <c r="F160" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="161" spans="1:6">
@@ -4495,7 +4519,7 @@
         <v>165</v>
       </c>
       <c r="B161" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C161">
         <v>0</v>
@@ -4507,7 +4531,7 @@
         <v>46298</v>
       </c>
       <c r="F161" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="162" spans="1:6">
@@ -4515,7 +4539,7 @@
         <v>166</v>
       </c>
       <c r="B162" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C162">
         <v>0</v>
@@ -4527,7 +4551,7 @@
         <v>46298</v>
       </c>
       <c r="F162" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="163" spans="1:6">
@@ -4535,7 +4559,7 @@
         <v>167</v>
       </c>
       <c r="B163" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C163">
         <v>0</v>
@@ -4547,7 +4571,7 @@
         <v>46298</v>
       </c>
       <c r="F163" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="164" spans="1:6">
@@ -4555,7 +4579,7 @@
         <v>168</v>
       </c>
       <c r="B164" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C164">
         <v>0</v>
@@ -4567,7 +4591,7 @@
         <v>46298</v>
       </c>
       <c r="F164" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="165" spans="1:6">
@@ -4575,7 +4599,7 @@
         <v>169</v>
       </c>
       <c r="B165" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C165">
         <v>0</v>
@@ -4587,7 +4611,7 @@
         <v>46298</v>
       </c>
       <c r="F165" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="166" spans="1:6">
@@ -4595,7 +4619,7 @@
         <v>170</v>
       </c>
       <c r="B166" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C166">
         <v>0</v>
@@ -4615,7 +4639,7 @@
         <v>144</v>
       </c>
       <c r="B167" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C167">
         <v>0</v>
@@ -4627,7 +4651,7 @@
         <v>46300</v>
       </c>
       <c r="F167" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="168" spans="1:6">
@@ -4635,7 +4659,7 @@
         <v>171</v>
       </c>
       <c r="B168" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C168">
         <v>0</v>
@@ -4647,7 +4671,7 @@
         <v>46300</v>
       </c>
       <c r="F168" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="169" spans="1:6">
@@ -4655,7 +4679,7 @@
         <v>172</v>
       </c>
       <c r="B169" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C169">
         <v>0</v>
@@ -4667,7 +4691,7 @@
         <v>46300</v>
       </c>
       <c r="F169" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="170" spans="1:6">
@@ -4675,7 +4699,7 @@
         <v>173</v>
       </c>
       <c r="B170" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C170">
         <v>0</v>
@@ -4687,7 +4711,7 @@
         <v>46300</v>
       </c>
       <c r="F170" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="171" spans="1:6">
@@ -4695,7 +4719,7 @@
         <v>174</v>
       </c>
       <c r="B171" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C171">
         <v>0</v>
@@ -4707,7 +4731,7 @@
         <v>46300</v>
       </c>
       <c r="F171" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="172" spans="1:6">
@@ -4715,7 +4739,7 @@
         <v>175</v>
       </c>
       <c r="B172" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C172">
         <v>0</v>
@@ -4727,7 +4751,7 @@
         <v>46300</v>
       </c>
       <c r="F172" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="173" spans="1:6">
@@ -4735,7 +4759,7 @@
         <v>176</v>
       </c>
       <c r="B173" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C173">
         <v>0</v>
@@ -4755,7 +4779,7 @@
         <v>177</v>
       </c>
       <c r="B174" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C174">
         <v>0</v>
@@ -4767,7 +4791,7 @@
         <v>46300</v>
       </c>
       <c r="F174" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="175" spans="1:6">
@@ -4775,7 +4799,7 @@
         <v>178</v>
       </c>
       <c r="B175" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C175">
         <v>0</v>
@@ -4787,7 +4811,67 @@
         <v>46300</v>
       </c>
       <c r="F175" t="s">
-        <v>327</v>
+        <v>334</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6">
+      <c r="A176" t="s">
+        <v>179</v>
+      </c>
+      <c r="B176" t="s">
+        <v>329</v>
+      </c>
+      <c r="C176">
+        <v>0</v>
+      </c>
+      <c r="D176" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E176" s="1">
+        <v>46300</v>
+      </c>
+      <c r="F176" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6">
+      <c r="A177" t="s">
+        <v>180</v>
+      </c>
+      <c r="B177" t="s">
+        <v>330</v>
+      </c>
+      <c r="C177">
+        <v>0</v>
+      </c>
+      <c r="D177" s="1">
+        <v>46300</v>
+      </c>
+      <c r="E177" s="1">
+        <v>46300</v>
+      </c>
+      <c r="F177" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6">
+      <c r="A178" t="s">
+        <v>181</v>
+      </c>
+      <c r="B178" t="s">
+        <v>331</v>
+      </c>
+      <c r="C178">
+        <v>0</v>
+      </c>
+      <c r="D178" t="s">
+        <v>332</v>
+      </c>
+      <c r="E178" t="s">
+        <v>332</v>
+      </c>
+      <c r="F178" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
automatic update 2026-10-07 08:49:03
</commit_message>
<xml_diff>
--- a/d_testing_folder/d_historical_test_results1.xlsx
+++ b/d_testing_folder/d_historical_test_results1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="354">
   <si>
     <t>Word</t>
   </si>
@@ -560,6 +560,33 @@
   </si>
   <si>
     <t>Posterior</t>
+  </si>
+  <si>
+    <t>FeatureAgglomeration</t>
+  </si>
+  <si>
+    <t>TfidfTransformer</t>
+  </si>
+  <si>
+    <t>SimCLR</t>
+  </si>
+  <si>
+    <t>TransformedTargetRegressor</t>
+  </si>
+  <si>
+    <t>Distribution Shape</t>
+  </si>
+  <si>
+    <t>Alan Kay 2</t>
+  </si>
+  <si>
+    <t>Austerity</t>
+  </si>
+  <si>
+    <t>Matthew 11:28:30</t>
+  </si>
+  <si>
+    <t>Proverbs 27:12</t>
   </si>
   <si>
     <t>A mathematical function applied to a neuron’s weighted input that introduces non-linearity into a neural network. This nonlinearity enables the model to learn complex, non-linear relationships in the data. Activation functions are applied within layers during the forward pass of a neural network, transforming intermediate representations before passing them to the next layer. Activation choice affects gradient flow, training stability, and convergence speed. Poor choices can cause vanishing or exploding gradients, limiting the depth or effectiveness of the network</t>
@@ -978,16 +1005,16 @@
     <t xml:space="preserve">Highest level in Organziational Taxonomy. Used to classify topics, concepts and ideas. While I have and continue to utilize a consistent nominclacture, it continues to evolve and expand. </t>
   </si>
   <si>
-    <t>{What the analytical method is: Expectation-Maximization (EM) is a statistical algorithm for finding maximum likelihood estimates of parameters in probabilistic models., How it works: The EM algorithm iteratively updates the model parameters and the unobserved variables until convergence, alternating between two steps: expectation (E-step) and maximization (M-step)., Why it is important: EM is essential for handling missing data and identifying underlying patterns in datasets. It is widely used in various applications, including clustering, classification, and dimensionality reduction., Its typical applications: EM is commonly employed in machine learning tasks such as cluster analysis, anomaly detection, and feature extraction.}</t>
-  </si>
-  <si>
-    <t>{What the analytical method is: As Features is a technique used to select relevant features from a dataset, often in the context of classification or regression problems., How it works: It typically involves evaluating the importance or relevance of each feature using various metrics such as mutual information, correlation coefficient, or recursive feature elimination (RFE), and selecting the top-ranked features for further analysis or modeling., Why it is important: Feature selection is crucial in machine learning to prevent overfitting, improve model interpretability, reduce dimensionality, and enhance prediction performance. By identifying the most relevant features, analysts can focus on the most informative variables and develop more accurate models., Its typical applications: As Features has been applied extensively in various domains such as text classification, image analysis, gene expression data analysis, and recommender systems.}</t>
-  </si>
-  <si>
-    <t>Autoencoding is a type of unsupervised learning algorithm that learns to compress and reconstruct input data., It works by defining an encoder network that maps the input data to a lower-dimensional latent space, and a decoder network that maps the latent space back to the original input data., The importance of autoencoding lies in its ability to learn compact representations of high-dimensional data, which can be useful for dimensionality reduction, anomaly detection, and generative modeling., Autoencoding is typically applied in areas such as image compression, text processing, and recommender systems.</t>
-  </si>
-  <si>
-    <t>MeanShift is a non-parametric, adaptive density-based clustering algorithm that automatically determines the number of clusters in the data. It works by iteratively shifting the centroids of overlapping Gaussian distributions towards higher-density regions until convergence. This method is important because it can handle complex, high-dimensional datasets and does not require any prior knowledge about the underlying structure. Typical applications include image segmentation, object tracking, and bioinformatics.</t>
+    <t>Expectation-Maximization (EM) is an iterative optimization algorithm for estimating parameters of probabilistic models when the data contain latent or unobserved variables, alternating between an Expectation (E) step that estimates the latent-variable distribution and a Maximization (M) step that updates model parameters. It is particularly relevant to problems such as Gaussian mixture model clustering, missing-data estimation, and other latent-variable models where direct maximum-likelihood estimation is difficult. EM is important because it transforms a difficult optimization involving hidden information into a sequence of more tractable estimation problems, with each iteration guaranteed not to decrease the observed-data likelihood under standard conditions. The general EM algorithm was formally named and popularized by Arthur Dempster, Nan Laird, and Donald Rubin in their influential 1977 paper, although related iterative estimation techniques existed earlier.</t>
+  </si>
+  <si>
+    <t>practice of transforming information, model outputs, or derived measurements into variables that serve as inputs to another statistical or machine-learning model. For example, cluster assignments, embeddings, predicted probabilities, dates, text-derived measurements, or aggregated historical behavior can all be represented as features for a downstream model. This approach is relevant to feature engineering, representation learning, ensemble methods, and multi-stage ML pipelines because it allows information discovered in one processing step to become predictive information for another. It is important because model performance often depends as much on how useful information is represented as features as on the choice of learning algorithm itself, although care must be taken to prevent problems such as target leakage.</t>
+  </si>
+  <si>
+    <t>Autoencoding is an unsupervised representation-learning technique in which a neural network learns to reconstruct its input after passing it through an intermediate latent representation, typically using an encoder and decoder. It is relevant when learning compact representations of high-dimensional data, particularly for dimensionality reduction, feature extraction, denoising, anomaly detection, and generative modeling. Autoencoding is important because the reconstruction objective allows useful features and structure to be learned from unlabeled data, while constraints such as a bottleneck, sparsity, or noise prevent the model from simply copying its input. Autoencoders developed from neural-network research into efficient data representations, with important early work appearing in the 1980s and later becoming prominent in deep learning through multilayer and variational architectures.</t>
+  </si>
+  <si>
+    <t>MeanShift is a non-parametric clustering algorithm that iteratively moves candidate cluster centers toward regions of higher estimated data density until they converge on local density modes. Unlike methods such as K-means, it does not require the number of clusters to be specified beforehand, but instead relies heavily on a bandwidth parameter that determines the neighborhood used for estimating density. It is relevant when clusters may have irregular distributions or when the appropriate number of clusters is unknown, although it can become computationally expensive for large or high-dimensional datasets. MeanShift originated in pattern-recognition research by Fukunaga and Hostetler in 1975 and was later popularized particularly in computer vision and image segmentation.</t>
   </si>
   <si>
     <t>Wherever your treasure is, there the desires of your heart will also be.</t>
@@ -1035,7 +1062,31 @@
     <t>A posterior probability or posterior distribution represents the probability assigned to an unknown parameter, hypothesis, or latent state after incorporating observed data or evidence. In Bayesian inference, the posterior is obtained by combining the prior distribution with the likelihood of the observed data according to Bayes' theorem and then normalizing the result. It therefore represents an updated state of knowledge given the available evidence. In a Gaussian Mixture Model, for example, the posterior component probabilities represent the estimated probabilities that a particular observation belongs to each Gaussian component after considering the observation's values.</t>
   </si>
   <si>
-    <t>2026-10-05</t>
+    <t>{What the analytical method is: FeatureAgglomeration is a technique used in machine learning to reduce the dimensionality of high-dimensional data., How it works: It works by merging similar features into a new feature, thereby reducing the number of features while retaining the most important information., Why it is important: This method is important because it can help prevent the curse of dimensionality and improve model interpretability., Its typical applications: FeatureAgglomeration is typically used in clustering, classification, and regression tasks where high-dimensional data is involved.}</t>
+  </si>
+  <si>
+    <t>{What the analytical method is: TfidfTransformer is a technique used to transform tokenized documents into numerical feature vectors., How it works: It calculates the importance of each word in the vocabulary by multiplying its frequency with its inverse document frequency (IDF)., Why it is important: This transformation helps in reducing the dimensionality of the data and highlights the importance of rare words, which can improve the performance of many machine learning algorithms., Its typical applications: TfidfTransformer is commonly used in natural language processing tasks such as text classification, sentiment analysis, and topic modeling.}</t>
+  </si>
+  <si>
+    <t>{What the analytical method is: SimCLR (Simultaneous Contrastive Learning of Representations) is a self-supervised learning algorithm that improves the representation capabilities of neural networks., How it works: It does this by maximizing agreement between different augmentations of the same input, while also minimizing agreement between different inputs., Why it is important: This allows SimCLR to learn robust and generalizable representations that can be used for various downstream tasks., Its typical applications: SimCLR has been successfully applied in various computer vision tasks, including image classification, object detection, and segmentation.}</t>
+  </si>
+  <si>
+    <t>TransformedTargetRegressor is a regression algorithm that uses a transformation of the target variable to improve the prediction accuracy. It works by first applying a transformation to the target variable, and then using a regressor to predict the transformed target variable. This method is important because it can handle non-linear relationships between the input features and the target variable, and can also be used for feature selection and dimensionality reduction. TransformedTargetRegressor is typically applied in regression tasks where the target variable has a non-linear relationship with the input features, such as predicting continuous outcomes like prices or scores.</t>
+  </si>
+  <si>
+    <t>Assess whether unusual distributional characteristics such as skewness, long tails, multimodality, or concentration are genuine characteristics of the population. Distributional characteristics may materially affect transformations, statistical measures, distance-based methods, and model selection.</t>
+  </si>
+  <si>
+    <t>The best way to predict the future is to invent it.</t>
+  </si>
+  <si>
+    <t>Extreme plainness and simplicity of style or appearance.</t>
+  </si>
+  <si>
+    <t>Come to me, all of you who are weary and carry heavy burdens, and I will give you rest. Take my yoke upon you. Let me teach you, because I am humble and gentle at heart, and you will find rest for your souls. For my yoke is easy to bear, and the burden I give you is light. (Matthew 11:28–30)</t>
+  </si>
+  <si>
+    <t>The prudent see danger and take refuge, but the simple keep going and pay the penalty.</t>
   </si>
   <si>
     <t>Concepts and Definitions</t>
@@ -1048,9 +1099,6 @@
   </si>
   <si>
     <t>Quote</t>
-  </si>
-  <si>
-    <t>Concepts And Definition</t>
   </si>
 </sst>
 </file>
@@ -1386,7 +1434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1414,7 +1462,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1426,7 +1474,7 @@
         <v>46023</v>
       </c>
       <c r="F2" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1434,7 +1482,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1446,7 +1494,7 @@
         <v>46023</v>
       </c>
       <c r="F3" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1454,7 +1502,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1466,7 +1514,7 @@
         <v>46023</v>
       </c>
       <c r="F4" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1474,7 +1522,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1486,7 +1534,7 @@
         <v>46023</v>
       </c>
       <c r="F5" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1503,7 +1551,7 @@
         <v>46023</v>
       </c>
       <c r="F6" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1511,7 +1559,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1523,7 +1571,7 @@
         <v>46023</v>
       </c>
       <c r="F7" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1531,7 +1579,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -1543,7 +1591,7 @@
         <v>46023</v>
       </c>
       <c r="F8" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1560,7 +1608,7 @@
         <v>46023</v>
       </c>
       <c r="F9" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1577,7 +1625,7 @@
         <v>46023</v>
       </c>
       <c r="F10" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1585,7 +1633,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1597,7 +1645,7 @@
         <v>46023</v>
       </c>
       <c r="F11" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1605,7 +1653,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1617,7 +1665,7 @@
         <v>46023</v>
       </c>
       <c r="F12" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1625,7 +1673,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1637,7 +1685,7 @@
         <v>46023</v>
       </c>
       <c r="F13" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1645,7 +1693,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1657,7 +1705,7 @@
         <v>46023</v>
       </c>
       <c r="F14" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1665,7 +1713,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1677,7 +1725,7 @@
         <v>46023</v>
       </c>
       <c r="F15" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1685,7 +1733,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1697,7 +1745,7 @@
         <v>46023</v>
       </c>
       <c r="F16" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1705,7 +1753,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1717,7 +1765,7 @@
         <v>46023</v>
       </c>
       <c r="F17" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1734,7 +1782,7 @@
         <v>46023</v>
       </c>
       <c r="F18" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1742,7 +1790,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1754,7 +1802,7 @@
         <v>46023</v>
       </c>
       <c r="F19" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1771,7 +1819,7 @@
         <v>46023</v>
       </c>
       <c r="F20" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1788,7 +1836,7 @@
         <v>46023</v>
       </c>
       <c r="F21" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1796,7 +1844,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1808,7 +1856,7 @@
         <v>46023</v>
       </c>
       <c r="F22" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1816,7 +1864,7 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1828,7 +1876,7 @@
         <v>46023</v>
       </c>
       <c r="F23" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1836,7 +1884,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -1848,7 +1896,7 @@
         <v>46023</v>
       </c>
       <c r="F24" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1865,7 +1913,7 @@
         <v>46023</v>
       </c>
       <c r="F25" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1882,7 +1930,7 @@
         <v>46023</v>
       </c>
       <c r="F26" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1890,7 +1938,7 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1902,7 +1950,7 @@
         <v>46023</v>
       </c>
       <c r="F27" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1919,7 +1967,7 @@
         <v>46023</v>
       </c>
       <c r="F28" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1927,7 +1975,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -1939,7 +1987,7 @@
         <v>46023</v>
       </c>
       <c r="F29" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1956,7 +2004,7 @@
         <v>46023</v>
       </c>
       <c r="F30" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1964,7 +2012,7 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1976,7 +2024,7 @@
         <v>46023</v>
       </c>
       <c r="F31" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1984,7 +2032,7 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -1996,7 +2044,7 @@
         <v>46023</v>
       </c>
       <c r="F32" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2013,7 +2061,7 @@
         <v>46023</v>
       </c>
       <c r="F33" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2021,7 +2069,7 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -2033,7 +2081,7 @@
         <v>46023</v>
       </c>
       <c r="F34" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2041,7 +2089,7 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -2053,7 +2101,7 @@
         <v>46023</v>
       </c>
       <c r="F35" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2070,7 +2118,7 @@
         <v>46023</v>
       </c>
       <c r="F36" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2078,7 +2126,7 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -2090,7 +2138,7 @@
         <v>46023</v>
       </c>
       <c r="F37" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2107,7 +2155,7 @@
         <v>46023</v>
       </c>
       <c r="F38" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2115,7 +2163,7 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -2127,7 +2175,7 @@
         <v>46023</v>
       </c>
       <c r="F39" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2135,7 +2183,7 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -2147,7 +2195,7 @@
         <v>46023</v>
       </c>
       <c r="F40" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2164,7 +2212,7 @@
         <v>46023</v>
       </c>
       <c r="F41" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2172,7 +2220,7 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -2184,7 +2232,7 @@
         <v>46296</v>
       </c>
       <c r="F42" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2192,7 +2240,7 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -2204,7 +2252,7 @@
         <v>46023</v>
       </c>
       <c r="F43" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -2212,7 +2260,7 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -2224,7 +2272,7 @@
         <v>46023</v>
       </c>
       <c r="F44" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -2232,7 +2280,7 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C45">
         <v>0</v>
@@ -2244,7 +2292,7 @@
         <v>46023</v>
       </c>
       <c r="F45" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -2252,7 +2300,7 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -2264,7 +2312,7 @@
         <v>46023</v>
       </c>
       <c r="F46" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2272,7 +2320,7 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -2284,7 +2332,7 @@
         <v>46023</v>
       </c>
       <c r="F47" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -2292,7 +2340,7 @@
         <v>52</v>
       </c>
       <c r="B48" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -2304,7 +2352,7 @@
         <v>46023</v>
       </c>
       <c r="F48" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -2321,7 +2369,7 @@
         <v>46023</v>
       </c>
       <c r="F49" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2329,7 +2377,7 @@
         <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -2341,7 +2389,7 @@
         <v>46023</v>
       </c>
       <c r="F50" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -2349,7 +2397,7 @@
         <v>55</v>
       </c>
       <c r="B51" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -2361,7 +2409,7 @@
         <v>46023</v>
       </c>
       <c r="F51" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2378,7 +2426,7 @@
         <v>46023</v>
       </c>
       <c r="F52" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2395,7 +2443,7 @@
         <v>46023</v>
       </c>
       <c r="F53" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2403,7 +2451,7 @@
         <v>58</v>
       </c>
       <c r="B54" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="C54">
         <v>0</v>
@@ -2415,7 +2463,7 @@
         <v>46023</v>
       </c>
       <c r="F54" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2423,7 +2471,7 @@
         <v>59</v>
       </c>
       <c r="B55" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="C55">
         <v>0</v>
@@ -2435,7 +2483,7 @@
         <v>46023</v>
       </c>
       <c r="F55" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2443,7 +2491,7 @@
         <v>60</v>
       </c>
       <c r="B56" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="C56">
         <v>0</v>
@@ -2455,7 +2503,7 @@
         <v>46023</v>
       </c>
       <c r="F56" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2472,7 +2520,7 @@
         <v>46023</v>
       </c>
       <c r="F57" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2480,7 +2528,7 @@
         <v>62</v>
       </c>
       <c r="B58" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="C58">
         <v>0</v>
@@ -2492,7 +2540,7 @@
         <v>46023</v>
       </c>
       <c r="F58" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2500,7 +2548,7 @@
         <v>63</v>
       </c>
       <c r="B59" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -2512,7 +2560,7 @@
         <v>46023</v>
       </c>
       <c r="F59" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2520,7 +2568,7 @@
         <v>64</v>
       </c>
       <c r="B60" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -2532,7 +2580,7 @@
         <v>46023</v>
       </c>
       <c r="F60" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -2540,7 +2588,7 @@
         <v>65</v>
       </c>
       <c r="B61" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -2552,7 +2600,7 @@
         <v>46296</v>
       </c>
       <c r="F61" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -2560,7 +2608,7 @@
         <v>66</v>
       </c>
       <c r="B62" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -2572,7 +2620,7 @@
         <v>46023</v>
       </c>
       <c r="F62" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -2580,7 +2628,7 @@
         <v>67</v>
       </c>
       <c r="B63" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -2592,7 +2640,7 @@
         <v>46023</v>
       </c>
       <c r="F63" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -2600,7 +2648,7 @@
         <v>68</v>
       </c>
       <c r="B64" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -2612,7 +2660,7 @@
         <v>46023</v>
       </c>
       <c r="F64" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -2620,7 +2668,7 @@
         <v>69</v>
       </c>
       <c r="B65" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -2632,7 +2680,7 @@
         <v>46023</v>
       </c>
       <c r="F65" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -2640,7 +2688,7 @@
         <v>70</v>
       </c>
       <c r="B66" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -2652,7 +2700,7 @@
         <v>46023</v>
       </c>
       <c r="F66" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -2660,7 +2708,7 @@
         <v>71</v>
       </c>
       <c r="B67" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C67">
         <v>0</v>
@@ -2672,7 +2720,7 @@
         <v>46296</v>
       </c>
       <c r="F67" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -2689,7 +2737,7 @@
         <v>46023</v>
       </c>
       <c r="F68" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -2697,7 +2745,7 @@
         <v>73</v>
       </c>
       <c r="B69" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -2709,7 +2757,7 @@
         <v>46023</v>
       </c>
       <c r="F69" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -2717,7 +2765,7 @@
         <v>74</v>
       </c>
       <c r="B70" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -2729,7 +2777,7 @@
         <v>46023</v>
       </c>
       <c r="F70" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -2737,7 +2785,7 @@
         <v>75</v>
       </c>
       <c r="B71" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -2749,7 +2797,7 @@
         <v>46023</v>
       </c>
       <c r="F71" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -2757,7 +2805,7 @@
         <v>76</v>
       </c>
       <c r="B72" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C72">
         <v>0</v>
@@ -2769,7 +2817,7 @@
         <v>46023</v>
       </c>
       <c r="F72" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -2786,7 +2834,7 @@
         <v>46023</v>
       </c>
       <c r="F73" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -2794,7 +2842,7 @@
         <v>78</v>
       </c>
       <c r="B74" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="C74">
         <v>0</v>
@@ -2806,7 +2854,7 @@
         <v>46023</v>
       </c>
       <c r="F74" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -2814,7 +2862,7 @@
         <v>79</v>
       </c>
       <c r="B75" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C75">
         <v>0</v>
@@ -2826,7 +2874,7 @@
         <v>46023</v>
       </c>
       <c r="F75" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -2843,7 +2891,7 @@
         <v>46023</v>
       </c>
       <c r="F76" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -2851,7 +2899,7 @@
         <v>81</v>
       </c>
       <c r="B77" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="C77">
         <v>0</v>
@@ -2863,7 +2911,7 @@
         <v>46023</v>
       </c>
       <c r="F77" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -2871,7 +2919,7 @@
         <v>82</v>
       </c>
       <c r="B78" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -2883,7 +2931,7 @@
         <v>46023</v>
       </c>
       <c r="F78" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -2891,7 +2939,7 @@
         <v>83</v>
       </c>
       <c r="B79" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -2903,7 +2951,7 @@
         <v>46023</v>
       </c>
       <c r="F79" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -2911,7 +2959,7 @@
         <v>84</v>
       </c>
       <c r="B80" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="C80">
         <v>0</v>
@@ -2923,7 +2971,7 @@
         <v>46023</v>
       </c>
       <c r="F80" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2931,7 +2979,7 @@
         <v>85</v>
       </c>
       <c r="B81" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="C81">
         <v>0</v>
@@ -2943,7 +2991,7 @@
         <v>46023</v>
       </c>
       <c r="F81" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2960,7 +3008,7 @@
         <v>46023</v>
       </c>
       <c r="F82" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -2968,7 +3016,7 @@
         <v>87</v>
       </c>
       <c r="B83" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="C83">
         <v>0</v>
@@ -2980,7 +3028,7 @@
         <v>46023</v>
       </c>
       <c r="F83" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2997,7 +3045,7 @@
         <v>46023</v>
       </c>
       <c r="F84" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -3005,7 +3053,7 @@
         <v>89</v>
       </c>
       <c r="B85" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -3017,7 +3065,7 @@
         <v>46023</v>
       </c>
       <c r="F85" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -3034,7 +3082,7 @@
         <v>46023</v>
       </c>
       <c r="F86" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -3051,7 +3099,7 @@
         <v>46023</v>
       </c>
       <c r="F87" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -3059,7 +3107,7 @@
         <v>92</v>
       </c>
       <c r="B88" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -3071,7 +3119,7 @@
         <v>46023</v>
       </c>
       <c r="F88" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -3079,7 +3127,7 @@
         <v>93</v>
       </c>
       <c r="B89" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -3091,7 +3139,7 @@
         <v>46023</v>
       </c>
       <c r="F89" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -3099,7 +3147,7 @@
         <v>94</v>
       </c>
       <c r="B90" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -3111,7 +3159,7 @@
         <v>46023</v>
       </c>
       <c r="F90" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -3119,7 +3167,7 @@
         <v>95</v>
       </c>
       <c r="B91" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -3131,7 +3179,7 @@
         <v>46023</v>
       </c>
       <c r="F91" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -3139,7 +3187,7 @@
         <v>96</v>
       </c>
       <c r="B92" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -3151,7 +3199,7 @@
         <v>46023</v>
       </c>
       <c r="F92" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -3159,7 +3207,7 @@
         <v>97</v>
       </c>
       <c r="B93" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -3171,7 +3219,7 @@
         <v>46023</v>
       </c>
       <c r="F93" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -3179,7 +3227,7 @@
         <v>98</v>
       </c>
       <c r="B94" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="C94">
         <v>0</v>
@@ -3191,7 +3239,7 @@
         <v>46023</v>
       </c>
       <c r="F94" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -3199,7 +3247,7 @@
         <v>99</v>
       </c>
       <c r="B95" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="C95">
         <v>0</v>
@@ -3211,7 +3259,7 @@
         <v>46023</v>
       </c>
       <c r="F95" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -3219,7 +3267,7 @@
         <v>100</v>
       </c>
       <c r="B96" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="C96">
         <v>0</v>
@@ -3231,7 +3279,7 @@
         <v>46296</v>
       </c>
       <c r="F96" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -3239,7 +3287,7 @@
         <v>101</v>
       </c>
       <c r="B97" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="C97">
         <v>0</v>
@@ -3251,7 +3299,7 @@
         <v>46023</v>
       </c>
       <c r="F97" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -3259,7 +3307,7 @@
         <v>102</v>
       </c>
       <c r="B98" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C98">
         <v>0</v>
@@ -3271,7 +3319,7 @@
         <v>46023</v>
       </c>
       <c r="F98" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3279,7 +3327,7 @@
         <v>103</v>
       </c>
       <c r="B99" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="C99">
         <v>0</v>
@@ -3291,7 +3339,7 @@
         <v>46023</v>
       </c>
       <c r="F99" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3299,7 +3347,7 @@
         <v>104</v>
       </c>
       <c r="B100" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="C100">
         <v>0</v>
@@ -3311,7 +3359,7 @@
         <v>46023</v>
       </c>
       <c r="F100" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -3319,7 +3367,7 @@
         <v>105</v>
       </c>
       <c r="B101" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="C101">
         <v>0</v>
@@ -3331,7 +3379,7 @@
         <v>46023</v>
       </c>
       <c r="F101" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3339,7 +3387,7 @@
         <v>106</v>
       </c>
       <c r="B102" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="C102">
         <v>0</v>
@@ -3351,7 +3399,7 @@
         <v>46023</v>
       </c>
       <c r="F102" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3359,7 +3407,7 @@
         <v>107</v>
       </c>
       <c r="B103" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="C103">
         <v>0</v>
@@ -3371,7 +3419,7 @@
         <v>46023</v>
       </c>
       <c r="F103" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3379,7 +3427,7 @@
         <v>108</v>
       </c>
       <c r="B104" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="C104">
         <v>0</v>
@@ -3391,7 +3439,7 @@
         <v>46296</v>
       </c>
       <c r="F104" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3399,7 +3447,7 @@
         <v>109</v>
       </c>
       <c r="B105" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="C105">
         <v>0</v>
@@ -3411,7 +3459,7 @@
         <v>46296</v>
       </c>
       <c r="F105" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3419,7 +3467,7 @@
         <v>110</v>
       </c>
       <c r="B106" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="C106">
         <v>0</v>
@@ -3431,7 +3479,7 @@
         <v>46023</v>
       </c>
       <c r="F106" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3439,7 +3487,7 @@
         <v>111</v>
       </c>
       <c r="B107" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C107">
         <v>0</v>
@@ -3451,7 +3499,7 @@
         <v>46023</v>
       </c>
       <c r="F107" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3459,7 +3507,7 @@
         <v>112</v>
       </c>
       <c r="B108" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -3471,7 +3519,7 @@
         <v>46023</v>
       </c>
       <c r="F108" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -3479,7 +3527,7 @@
         <v>113</v>
       </c>
       <c r="B109" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -3491,7 +3539,7 @@
         <v>46296</v>
       </c>
       <c r="F109" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3499,7 +3547,7 @@
         <v>114</v>
       </c>
       <c r="B110" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -3511,7 +3559,7 @@
         <v>46023</v>
       </c>
       <c r="F110" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -3519,7 +3567,7 @@
         <v>115</v>
       </c>
       <c r="B111" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -3531,7 +3579,7 @@
         <v>46023</v>
       </c>
       <c r="F111" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3539,7 +3587,7 @@
         <v>116</v>
       </c>
       <c r="B112" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -3551,7 +3599,7 @@
         <v>46296</v>
       </c>
       <c r="F112" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -3559,7 +3607,7 @@
         <v>117</v>
       </c>
       <c r="B113" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -3579,7 +3627,7 @@
         <v>118</v>
       </c>
       <c r="B114" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -3599,7 +3647,7 @@
         <v>119</v>
       </c>
       <c r="B115" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -3619,7 +3667,7 @@
         <v>120</v>
       </c>
       <c r="B116" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="C116">
         <v>0</v>
@@ -3639,7 +3687,7 @@
         <v>121</v>
       </c>
       <c r="B117" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="C117">
         <v>0</v>
@@ -3659,7 +3707,7 @@
         <v>122</v>
       </c>
       <c r="B118" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="C118">
         <v>0</v>
@@ -3679,7 +3727,7 @@
         <v>123</v>
       </c>
       <c r="B119" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="C119">
         <v>0</v>
@@ -3699,7 +3747,7 @@
         <v>124</v>
       </c>
       <c r="B120" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C120">
         <v>0</v>
@@ -3719,7 +3767,7 @@
         <v>125</v>
       </c>
       <c r="B121" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="C121">
         <v>0</v>
@@ -3739,7 +3787,7 @@
         <v>126</v>
       </c>
       <c r="B122" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C122">
         <v>0</v>
@@ -3751,7 +3799,7 @@
         <v>46296</v>
       </c>
       <c r="F122" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -3759,7 +3807,7 @@
         <v>127</v>
       </c>
       <c r="B123" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="C123">
         <v>0</v>
@@ -3771,7 +3819,7 @@
         <v>46296</v>
       </c>
       <c r="F123" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -3779,7 +3827,7 @@
         <v>128</v>
       </c>
       <c r="B124" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="C124">
         <v>0</v>
@@ -3791,7 +3839,7 @@
         <v>46023</v>
       </c>
       <c r="F124" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -3799,7 +3847,7 @@
         <v>129</v>
       </c>
       <c r="B125" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="C125">
         <v>0</v>
@@ -3811,7 +3859,7 @@
         <v>46296</v>
       </c>
       <c r="F125" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -3819,7 +3867,7 @@
         <v>130</v>
       </c>
       <c r="B126" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="C126">
         <v>0</v>
@@ -3831,7 +3879,7 @@
         <v>46023</v>
       </c>
       <c r="F126" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -3839,7 +3887,7 @@
         <v>131</v>
       </c>
       <c r="B127" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="C127">
         <v>0</v>
@@ -3851,7 +3899,7 @@
         <v>46023</v>
       </c>
       <c r="F127" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -3859,7 +3907,7 @@
         <v>132</v>
       </c>
       <c r="B128" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="C128">
         <v>0</v>
@@ -3871,7 +3919,7 @@
         <v>46023</v>
       </c>
       <c r="F128" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -3879,7 +3927,7 @@
         <v>133</v>
       </c>
       <c r="B129" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C129">
         <v>0</v>
@@ -3891,7 +3939,7 @@
         <v>46023</v>
       </c>
       <c r="F129" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -3899,7 +3947,7 @@
         <v>134</v>
       </c>
       <c r="B130" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="C130">
         <v>0</v>
@@ -3911,7 +3959,7 @@
         <v>46023</v>
       </c>
       <c r="F130" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -3919,7 +3967,7 @@
         <v>135</v>
       </c>
       <c r="B131" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="C131">
         <v>0</v>
@@ -3931,7 +3979,7 @@
         <v>46023</v>
       </c>
       <c r="F131" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -3939,7 +3987,7 @@
         <v>136</v>
       </c>
       <c r="B132" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="C132">
         <v>0</v>
@@ -3951,7 +3999,7 @@
         <v>46023</v>
       </c>
       <c r="F132" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -3959,7 +4007,7 @@
         <v>137</v>
       </c>
       <c r="B133" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="C133">
         <v>0</v>
@@ -3971,7 +4019,7 @@
         <v>46023</v>
       </c>
       <c r="F133" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -3979,7 +4027,7 @@
         <v>138</v>
       </c>
       <c r="B134" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -3991,7 +4039,7 @@
         <v>46023</v>
       </c>
       <c r="F134" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -3999,7 +4047,7 @@
         <v>139</v>
       </c>
       <c r="B135" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -4011,7 +4059,7 @@
         <v>46023</v>
       </c>
       <c r="F135" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -4019,7 +4067,7 @@
         <v>140</v>
       </c>
       <c r="B136" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -4039,7 +4087,7 @@
         <v>141</v>
       </c>
       <c r="B137" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -4059,7 +4107,7 @@
         <v>142</v>
       </c>
       <c r="B138" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -4071,7 +4119,7 @@
         <v>46023</v>
       </c>
       <c r="F138" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="139" spans="1:6">
@@ -4079,7 +4127,7 @@
         <v>143</v>
       </c>
       <c r="B139" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="C139">
         <v>0</v>
@@ -4099,7 +4147,7 @@
         <v>144</v>
       </c>
       <c r="B140" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -4111,7 +4159,7 @@
         <v>46295</v>
       </c>
       <c r="F140" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="141" spans="1:6">
@@ -4119,7 +4167,7 @@
         <v>145</v>
       </c>
       <c r="B141" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -4131,7 +4179,7 @@
         <v>46295</v>
       </c>
       <c r="F141" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -4139,7 +4187,7 @@
         <v>146</v>
       </c>
       <c r="B142" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -4151,7 +4199,7 @@
         <v>46295</v>
       </c>
       <c r="F142" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -4159,7 +4207,7 @@
         <v>147</v>
       </c>
       <c r="B143" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="C143">
         <v>0</v>
@@ -4171,7 +4219,7 @@
         <v>46295</v>
       </c>
       <c r="F143" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -4179,7 +4227,7 @@
         <v>148</v>
       </c>
       <c r="B144" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="C144">
         <v>0</v>
@@ -4191,7 +4239,7 @@
         <v>46295</v>
       </c>
       <c r="F144" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="145" spans="1:6">
@@ -4199,7 +4247,7 @@
         <v>149</v>
       </c>
       <c r="B145" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C145">
         <v>0</v>
@@ -4211,7 +4259,7 @@
         <v>46295</v>
       </c>
       <c r="F145" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -4219,7 +4267,7 @@
         <v>150</v>
       </c>
       <c r="B146" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="C146">
         <v>0</v>
@@ -4231,7 +4279,7 @@
         <v>46296</v>
       </c>
       <c r="F146" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="147" spans="1:6">
@@ -4239,7 +4287,7 @@
         <v>151</v>
       </c>
       <c r="B147" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="C147">
         <v>0</v>
@@ -4251,7 +4299,7 @@
         <v>46295</v>
       </c>
       <c r="F147" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="148" spans="1:6">
@@ -4259,7 +4307,7 @@
         <v>152</v>
       </c>
       <c r="B148" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="C148">
         <v>0</v>
@@ -4279,7 +4327,7 @@
         <v>153</v>
       </c>
       <c r="B149" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -4291,7 +4339,7 @@
         <v>46296</v>
       </c>
       <c r="F149" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="150" spans="1:6">
@@ -4299,7 +4347,7 @@
         <v>154</v>
       </c>
       <c r="B150" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="C150">
         <v>0</v>
@@ -4311,7 +4359,7 @@
         <v>46296</v>
       </c>
       <c r="F150" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="151" spans="1:6">
@@ -4319,7 +4367,7 @@
         <v>155</v>
       </c>
       <c r="B151" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="C151">
         <v>0</v>
@@ -4331,7 +4379,7 @@
         <v>46296</v>
       </c>
       <c r="F151" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="152" spans="1:6">
@@ -4339,7 +4387,7 @@
         <v>156</v>
       </c>
       <c r="B152" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="C152">
         <v>0</v>
@@ -4351,7 +4399,7 @@
         <v>46296</v>
       </c>
       <c r="F152" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="153" spans="1:6">
@@ -4359,7 +4407,7 @@
         <v>157</v>
       </c>
       <c r="B153" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="C153">
         <v>0</v>
@@ -4371,7 +4419,7 @@
         <v>46296</v>
       </c>
       <c r="F153" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="154" spans="1:6">
@@ -4379,7 +4427,7 @@
         <v>158</v>
       </c>
       <c r="B154" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="C154">
         <v>0</v>
@@ -4399,7 +4447,7 @@
         <v>159</v>
       </c>
       <c r="B155" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="C155">
         <v>0</v>
@@ -4411,7 +4459,7 @@
         <v>46296</v>
       </c>
       <c r="F155" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -4419,7 +4467,7 @@
         <v>160</v>
       </c>
       <c r="B156" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -4431,7 +4479,7 @@
         <v>46296</v>
       </c>
       <c r="F156" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="157" spans="1:6">
@@ -4439,7 +4487,7 @@
         <v>161</v>
       </c>
       <c r="B157" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="C157">
         <v>0</v>
@@ -4451,7 +4499,7 @@
         <v>46296</v>
       </c>
       <c r="F157" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="158" spans="1:6">
@@ -4459,7 +4507,7 @@
         <v>162</v>
       </c>
       <c r="B158" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -4471,7 +4519,7 @@
         <v>46298</v>
       </c>
       <c r="F158" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="159" spans="1:6">
@@ -4479,7 +4527,7 @@
         <v>163</v>
       </c>
       <c r="B159" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -4491,7 +4539,7 @@
         <v>46298</v>
       </c>
       <c r="F159" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="160" spans="1:6">
@@ -4499,7 +4547,7 @@
         <v>164</v>
       </c>
       <c r="B160" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
       <c r="C160">
         <v>0</v>
@@ -4511,7 +4559,7 @@
         <v>46298</v>
       </c>
       <c r="F160" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="161" spans="1:6">
@@ -4519,7 +4567,7 @@
         <v>165</v>
       </c>
       <c r="B161" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="C161">
         <v>0</v>
@@ -4531,7 +4579,7 @@
         <v>46298</v>
       </c>
       <c r="F161" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="162" spans="1:6">
@@ -4539,7 +4587,7 @@
         <v>166</v>
       </c>
       <c r="B162" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="C162">
         <v>0</v>
@@ -4551,7 +4599,7 @@
         <v>46298</v>
       </c>
       <c r="F162" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="163" spans="1:6">
@@ -4559,7 +4607,7 @@
         <v>167</v>
       </c>
       <c r="B163" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C163">
         <v>0</v>
@@ -4571,7 +4619,7 @@
         <v>46298</v>
       </c>
       <c r="F163" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
     </row>
     <row r="164" spans="1:6">
@@ -4579,7 +4627,7 @@
         <v>168</v>
       </c>
       <c r="B164" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="C164">
         <v>0</v>
@@ -4591,7 +4639,7 @@
         <v>46298</v>
       </c>
       <c r="F164" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
     </row>
     <row r="165" spans="1:6">
@@ -4599,7 +4647,7 @@
         <v>169</v>
       </c>
       <c r="B165" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="C165">
         <v>0</v>
@@ -4611,7 +4659,7 @@
         <v>46298</v>
       </c>
       <c r="F165" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
     </row>
     <row r="166" spans="1:6">
@@ -4619,7 +4667,7 @@
         <v>170</v>
       </c>
       <c r="B166" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="C166">
         <v>0</v>
@@ -4636,10 +4684,10 @@
     </row>
     <row r="167" spans="1:6">
       <c r="A167" t="s">
-        <v>144</v>
+        <v>171</v>
       </c>
       <c r="B167" t="s">
-        <v>294</v>
+        <v>330</v>
       </c>
       <c r="C167">
         <v>0</v>
@@ -4651,15 +4699,15 @@
         <v>46300</v>
       </c>
       <c r="F167" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="168" spans="1:6">
       <c r="A168" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B168" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="C168">
         <v>0</v>
@@ -4671,15 +4719,15 @@
         <v>46300</v>
       </c>
       <c r="F168" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="169" spans="1:6">
       <c r="A169" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B169" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="C169">
         <v>0</v>
@@ -4691,15 +4739,15 @@
         <v>46300</v>
       </c>
       <c r="F169" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="170" spans="1:6">
       <c r="A170" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B170" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
       <c r="C170">
         <v>0</v>
@@ -4711,15 +4759,15 @@
         <v>46300</v>
       </c>
       <c r="F170" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
     </row>
     <row r="171" spans="1:6">
       <c r="A171" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B171" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="C171">
         <v>0</v>
@@ -4731,15 +4779,15 @@
         <v>46300</v>
       </c>
       <c r="F171" t="s">
-        <v>333</v>
+        <v>353</v>
       </c>
     </row>
     <row r="172" spans="1:6">
       <c r="A172" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B172" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="C172">
         <v>0</v>
@@ -4751,15 +4799,15 @@
         <v>46300</v>
       </c>
       <c r="F172" t="s">
-        <v>336</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:6">
       <c r="A173" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B173" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="C173">
         <v>0</v>
@@ -4771,15 +4819,15 @@
         <v>46300</v>
       </c>
       <c r="F173" t="s">
-        <v>0</v>
+        <v>352</v>
       </c>
     </row>
     <row r="174" spans="1:6">
       <c r="A174" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B174" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="C174">
         <v>0</v>
@@ -4791,15 +4839,15 @@
         <v>46300</v>
       </c>
       <c r="F174" t="s">
-        <v>335</v>
+        <v>351</v>
       </c>
     </row>
     <row r="175" spans="1:6">
       <c r="A175" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B175" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C175">
         <v>0</v>
@@ -4811,15 +4859,15 @@
         <v>46300</v>
       </c>
       <c r="F175" t="s">
-        <v>334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176" spans="1:6">
       <c r="A176" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B176" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="C176">
         <v>0</v>
@@ -4831,15 +4879,15 @@
         <v>46300</v>
       </c>
       <c r="F176" t="s">
-        <v>0</v>
+        <v>350</v>
       </c>
     </row>
     <row r="177" spans="1:6">
       <c r="A177" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B177" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C177">
         <v>0</v>
@@ -4851,27 +4899,187 @@
         <v>46300</v>
       </c>
       <c r="F177" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
     </row>
     <row r="178" spans="1:6">
       <c r="A178" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B178" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="C178">
         <v>0</v>
       </c>
-      <c r="D178" t="s">
-        <v>332</v>
-      </c>
-      <c r="E178" t="s">
-        <v>332</v>
+      <c r="D178" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E178" s="1">
+        <v>46301</v>
       </c>
       <c r="F178" t="s">
-        <v>337</v>
+        <v>350</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6">
+      <c r="A179" t="s">
+        <v>183</v>
+      </c>
+      <c r="B179" t="s">
+        <v>342</v>
+      </c>
+      <c r="C179">
+        <v>0</v>
+      </c>
+      <c r="D179" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E179" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F179" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6">
+      <c r="A180" t="s">
+        <v>184</v>
+      </c>
+      <c r="B180" t="s">
+        <v>343</v>
+      </c>
+      <c r="C180">
+        <v>0</v>
+      </c>
+      <c r="D180" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E180" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F180" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6">
+      <c r="A181" t="s">
+        <v>185</v>
+      </c>
+      <c r="B181" t="s">
+        <v>344</v>
+      </c>
+      <c r="C181">
+        <v>0</v>
+      </c>
+      <c r="D181" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E181" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F181" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6">
+      <c r="A182" t="s">
+        <v>186</v>
+      </c>
+      <c r="B182" t="s">
+        <v>345</v>
+      </c>
+      <c r="C182">
+        <v>0</v>
+      </c>
+      <c r="D182" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E182" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F182" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6">
+      <c r="A183" t="s">
+        <v>187</v>
+      </c>
+      <c r="B183" t="s">
+        <v>346</v>
+      </c>
+      <c r="C183">
+        <v>0</v>
+      </c>
+      <c r="D183" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E183" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F183" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6">
+      <c r="A184" t="s">
+        <v>188</v>
+      </c>
+      <c r="B184" t="s">
+        <v>347</v>
+      </c>
+      <c r="C184">
+        <v>0</v>
+      </c>
+      <c r="D184" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E184" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F184" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6">
+      <c r="A185" t="s">
+        <v>189</v>
+      </c>
+      <c r="B185" t="s">
+        <v>348</v>
+      </c>
+      <c r="C185">
+        <v>0</v>
+      </c>
+      <c r="D185" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E185" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F185" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6">
+      <c r="A186" t="s">
+        <v>190</v>
+      </c>
+      <c r="B186" t="s">
+        <v>349</v>
+      </c>
+      <c r="C186">
+        <v>0</v>
+      </c>
+      <c r="D186" s="1">
+        <v>46301</v>
+      </c>
+      <c r="E186" s="1">
+        <v>46301</v>
+      </c>
+      <c r="F186" t="s">
+        <v>352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>